<commit_message>
Fichas por classe, tier das incursoes e bando por combate
Seis mudancas que se acumularam no playtest:

- Ficha por classe: o jogador escolhe uma das 7 classes com tabela e as
  pericias com proficiencia; HP, CA, acerto, dano e bonus saem do tier e
  nao ficam gravados. Todo personagem comeca no nivel 1 e sobe com
  /ficha upar, ate o 10. Sai /ficha atributo, /ficha combate e /ficha nivel.
- Tier das incursoes: entra quem for do tier da incursao ou abaixo.
- Intervalo semanal com virada na segunda, em vez de 7 dias corridos.
- Caminho sorteado passo a passo: sala visitada nao volta a ser oferecida.
- Varias criaturas por combate, com menu de alvo e revide de cada uma.
- Retratos do grupo lado a lado na abertura da run (Pillow).

Fichas antigas nao tem como virar ficha nova (sem classe, sem numeros):
a migracao apaga os personagens e encerra as runs que dependiam deles.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/planilhas/banco_vortice_oculto.xlsx
+++ b/data/planilhas/banco_vortice_oculto.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Leia-me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Banco" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Salas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dificuldades" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pericias" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Monstros" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dificuldades" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Pericias" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -109,8 +110,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -245,32 +246,82 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
+        <t>Quantas criaturas iguais. Vazio ou 1 = uma. Máximo 6 por sala, contando as da aba 'Monstros'.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
         <t>Classe de Armadura do monstro.</t>
       </text>
     </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
+    <comment ref="M1" authorId="0" shapeId="0">
       <text>
         <t>Bônus de ataque do monstro (ex.: 6).</t>
       </text>
     </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
+    <comment ref="N1" authorId="0" shapeId="0">
       <text>
         <t>Dado de dano do monstro (ex.: 2d6+3).</t>
       </text>
     </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
+    <comment ref="O1" authorId="0" shapeId="0">
       <text>
         <t>Pontos de vida do monstro.</t>
       </text>
     </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
+    <comment ref="P1" authorId="0" shapeId="0">
       <text>
         <t>Bônus da sala (texto livre). Opcional.</t>
       </text>
     </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
+    <comment ref="Q1" authorId="0" shapeId="0">
       <text>
         <t>Pontos de Organizacao se a sala for superada. 0 ou vazio = nenhum.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Incursoes 2.0</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Criaturas EXTRAS de uma sala, para um bando misto. O que estiver aqui se soma ao monstro_* da linha da sala, ate 6 criaturas por sala. Deixe a aba vazia se cada sala tiver so um tipo de criatura.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Nome da criatura.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Quantas iguais. Vazio ou 1 = uma.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Classe de Armadura.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Bonus de ataque (ex.: 4).</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Dado de dano (ex.: 1d6+2).</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Pontos de vida de cada uma.</t>
       </text>
     </comment>
   </commentList>
@@ -768,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -781,12 +832,13 @@
     <col width="62" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="32" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="32" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -842,30 +894,35 @@
       </c>
       <c r="K1" s="4" t="inlineStr">
         <is>
+          <t>monstro_quantidade</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
           <t>monstro_ca</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>monstro_ataque</t>
         </is>
       </c>
-      <c r="M1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>monstro_dano</t>
         </is>
       </c>
-      <c r="N1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>monstro_hp</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>recompensa</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>pontos_organizacao</t>
         </is>
@@ -912,16 +969,17 @@
       </c>
       <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="5" t="inlineStr"/>
-      <c r="K2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="n"/>
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr"/>
       <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr"/>
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>Um fragmento de selo para quem passa ileso.</t>
         </is>
       </c>
-      <c r="P2" s="5" t="n">
+      <c r="Q2" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -966,16 +1024,17 @@
       </c>
       <c r="I3" s="5" t="inlineStr"/>
       <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="n"/>
       <c r="L3" s="5" t="inlineStr"/>
       <c r="M3" s="5" t="inlineStr"/>
       <c r="N3" s="5" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Revela a CA do próximo inimigo.</t>
         </is>
       </c>
-      <c r="P3" s="5" t="n">
+      <c r="Q3" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1017,21 +1076,24 @@
         </is>
       </c>
       <c r="K4" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="M4" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>1d10+3</t>
         </is>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="O4" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="n">
+      <c r="P4" s="5" t="inlineStr"/>
+      <c r="Q4" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1076,12 +1138,13 @@
       </c>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="n"/>
       <c r="L5" s="5" t="inlineStr"/>
       <c r="M5" s="5" t="inlineStr"/>
       <c r="N5" s="5" t="inlineStr"/>
       <c r="O5" s="5" t="inlineStr"/>
-      <c r="P5" s="5" t="n">
+      <c r="P5" s="5" t="inlineStr"/>
+      <c r="Q5" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1118,16 +1181,17 @@
       </c>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr"/>
-      <c r="K6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="n"/>
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr"/>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>O grupo recupera o fôlego.</t>
         </is>
       </c>
-      <c r="P6" s="5" t="n">
+      <c r="Q6" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1172,16 +1236,17 @@
       </c>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="n"/>
       <c r="L7" s="5" t="inlineStr"/>
       <c r="M7" s="5" t="inlineStr"/>
       <c r="N7" s="5" t="inlineStr"/>
-      <c r="O7" s="5" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr"/>
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>Materiais raros para quem passar no teste.</t>
         </is>
       </c>
-      <c r="P7" s="5" t="n">
+      <c r="Q7" s="5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1222,22 +1287,23 @@
           <t>Cria do Vazio</t>
         </is>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="M8" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>2d6+2</t>
         </is>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="O8" s="5" t="n">
         <v>34</v>
       </c>
-      <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="n">
+      <c r="P8" s="5" t="inlineStr"/>
+      <c r="Q8" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1282,16 +1348,17 @@
       </c>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="n"/>
       <c r="L9" s="5" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr"/>
       <c r="N9" s="5" t="inlineStr"/>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr"/>
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>O chefe começa o confronto final com 10 de HP a menos.</t>
         </is>
       </c>
-      <c r="P9" s="5" t="n">
+      <c r="Q9" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1336,12 +1403,13 @@
       </c>
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr"/>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="n"/>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
-      <c r="P10" s="5" t="n">
+      <c r="P10" s="5" t="inlineStr"/>
+      <c r="Q10" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1386,16 +1454,17 @@
       </c>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="inlineStr"/>
+      <c r="K11" s="5" t="n"/>
       <c r="L11" s="5" t="inlineStr"/>
       <c r="M11" s="5" t="inlineStr"/>
       <c r="N11" s="5" t="inlineStr"/>
-      <c r="O11" s="5" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr"/>
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>Atalho: a próxima sala começa com metade do progresso feito.</t>
         </is>
       </c>
-      <c r="P11" s="5" t="n">
+      <c r="Q11" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1436,22 +1505,23 @@
           <t>Coisa do Umbral</t>
         </is>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="L12" s="5" t="n">
+      <c r="M12" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>2d8+3</t>
         </is>
       </c>
-      <c r="N12" s="5" t="n">
+      <c r="O12" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="O12" s="5" t="inlineStr"/>
-      <c r="P12" s="5" t="n">
+      <c r="P12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1496,16 +1566,17 @@
       </c>
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="n"/>
       <c r="L13" s="5" t="inlineStr"/>
       <c r="M13" s="5" t="inlineStr"/>
       <c r="N13" s="5" t="inlineStr"/>
-      <c r="O13" s="5" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr"/>
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>Um item mágico menor, a critério do GM.</t>
         </is>
       </c>
-      <c r="P13" s="5" t="n">
+      <c r="Q13" s="5" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1529,6 +1600,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>sala_id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>quantidade</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>ca</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>ataque</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>dano</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>VO11</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Larva do Umbral</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>1d6</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1538,58 +1699,58 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>dificuldade</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>cd</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="8" t="inlineStr">
         <is>
           <t>alvo_progresso</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="7" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Média</t>
         </is>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="7" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Difícil</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="7" t="n">
         <v>15</v>
       </c>
     </row>
@@ -1605,7 +1766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1619,12 +1780,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>perícia</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="8" t="inlineStr">
         <is>
           <t>atributo</t>
         </is>

</xml_diff>

<commit_message>
Duas salas novas no banco do Vortice Oculto
VO13 Oficina de Ambar (dois Golens Menores e o Golem de Ambar) e VO14
Necroterio do Selo (tres Zumbis Putrefatos e o Necromante Mestre): as quatro
criaturas novas, ja com multiataque, vantagem em save e a acao especial.

As colunas novas entraram na aba Monstros da planilha, que continua sendo a
fonte — o JSON saiu do importador.

O simulador tambem passou a aceitar o JSON de um banco (--sala VO13), e a
levar em conta o multiataque, os saves e o atordoamento da criatura.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/planilhas/banco_vortice_oculto.xlsx
+++ b/data/planilhas/banco_vortice_oculto.xlsx
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,6 +112,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -322,6 +325,61 @@
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Pontos de vida de cada uma.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Golpes por rodada (multiataque). Vazio ou 1 = um.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Resistencias da criatura: 'FOR +5, CON +5'. O que faltar o bot deduz do bonus de ataque.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Atributos em que ela resiste com vantagem: 'FOR, CON'.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Nome da acao especial. Vazio = a criatura so ataca.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Descricao mostrada ao grupo. Opcional.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Atributo que os alvos rolam: FOR, DES, CON, INT, SAB ou CAR.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>CD do teste de resistencia (ex.: 13).</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Dano de quem falhar (ex.: 3d6). Vazio = so o efeito.</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>Quantos personagens ela pega de uma vez. Vazio = 1.</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Rodadas de atordoamento em quem falhar. Vazio ou 0 = nenhuma.</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>De quantas em quantas rodadas ela usa. Vazio = 2 (rodadas 2, 4, 6...). Na rodada que usa, ela nao ataca.</t>
       </text>
     </comment>
   </commentList>
@@ -819,7 +877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1580,6 +1638,88 @@
         <v>3</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>VO13</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Oficina de Âmbar</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Combate</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Resina antiga escorre das paredes e endurece antes de chegar ao chão. No meio da sala, três formas de pedra e âmbar esperam de pé — e a maior delas abre os olhos quando a porta range.</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="5" t="n"/>
+      <c r="O14" s="5" t="n"/>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>Um naco de âmbar ainda morno, que guarda alguma coisa dentro.</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>VO14</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Necrotério do Selo</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Combate</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="9" t="n"/>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Alguém chegou ao selo antes do grupo e não veio sozinho: trouxe os mortos da própria escavação. O necromante nem se vira — continua trabalhando enquanto o que sobrou deles caminha na direção da porta.</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="5" t="n"/>
+      <c r="O15" s="5" t="n"/>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>As anotações do necromante sobre o selo.</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -1600,7 +1740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1610,6 +1750,17 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1648,6 +1799,61 @@
           <t>hp</t>
         </is>
       </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>ataques</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>saves</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>saves_vantagem</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_texto</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_save</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_cd</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_dano</t>
+        </is>
+      </c>
+      <c r="P1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_alvos</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_atordoa</t>
+        </is>
+      </c>
+      <c r="R1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_cada</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
@@ -1676,6 +1882,218 @@
       </c>
       <c r="G2" s="7" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>VO13</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Golem Menor</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1d8+3</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>FOR, CON</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>VO13</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Golem de Âmbar</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1d8+4</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Prisão de Âmbar</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Uma explosão de âmbar prende quem não resistir.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>VO14</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Zumbi Putrefato</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1d6+1</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="n"/>
+      <c r="R5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>VO14</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Necromante Mestre</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1d8+3</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Explosão de Agonia</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Uma onda de energia sombria varre dois alvos de uma vez.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>DES</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>3d6</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Medusa e Nothic: recharge, save que se repete e dano somado
Tres mecanicas novas, pedidas pelo bloco da Medusa:

- Recharge 5-6: a habilidade sai carregada, e depois de gasta so volta quando
  o d6 da criatura tirar o numero da recarga. A carga fica no banco, entao um
  restart no meio do combate nao devolve o olhar de graca
- "refazem o save no final do turno": o atordoamento deixou de ter prazo fixo
  e passou a acabar quando o alvo passa no teste, no fim da rodada — sempre
  depois de perder ao menos uma vez
- dano em parcelas: "3d8+3+2d6" num campo so, para o golpe que corta e
  envenena. No critico os dados dobram e os numeros soltos entram uma vez

E a sala VO15 Jardim de Estatuas no banco do Vortice Oculto: tres Nothics e a
Medusa. O simulador entende as tres coisas e mostra a recarga no cabecalho.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/planilhas/banco_vortice_oculto.xlsx
+++ b/data/planilhas/banco_vortice_oculto.xlsx
@@ -380,6 +380,16 @@
     <comment ref="R1" authorId="0" shapeId="0">
       <text>
         <t>De quantas em quantas rodadas ela usa. Vazio = 2 (rodadas 2, 4, 6...). Na rodada que usa, ela nao ataca.</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>Recharge da 5e: a menor face do d6 que recarrega. 'Recharge 5-6' = 5. Com isto, 'cada' nao vale: sai na rodada 1 e depois volta quando o dado deixar.</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>x = o alvo refaz o save no fim de cada turno e se livra quando passar. Vazio = dura as rodadas de 'atordoa'.</t>
       </text>
     </comment>
   </commentList>
@@ -877,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1720,6 +1730,47 @@
         <v>3</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>VO15</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Jardim de Estátuas</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Combate</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="9" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>As figuras de pedra no corredor estão em posições erradas: uma protege o rosto, outra corre. No fundo, algo se arrasta sobre a própria cauda e três vultos magros se levantam das sombras, farejando.</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="5" t="n"/>
+      <c r="O16" s="5" t="n"/>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>O que a última estátua ainda segurava na mão.</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -1740,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1761,6 +1812,8 @@
     <col width="15" customWidth="1" min="16" max="16"/>
     <col width="17" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1852,6 +1905,16 @@
       <c r="R1" s="4" t="inlineStr">
         <is>
           <t>habilidade_cada</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_recarga</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>habilidade_save_repete</t>
         </is>
       </c>
     </row>
@@ -2094,6 +2157,114 @@
       </c>
       <c r="R6" s="2" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>VO15</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Nothic</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1d10+3</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>VO15</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Medusa</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>3d8+3+2d6</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>172</v>
+      </c>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Petrifying Gaze</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>O olhar endurece quem cruzar com ele.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="O8" s="2" t="n"/>
+      <c r="P8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
A Medusa vira o chefe da dungeon de teste, olhando todo mundo
O Petrifying Gaze pega o grupo inteiro (alvos 6), como manda o bloco dela.

A Cripta do Vortice passou a terminar na Medusa com tres Nothics de escolta,
no lugar do Guardiao do Selo generico do modelo — o combate garantido da run,
que e onde a recarga e o save-no-fim-do-turno aparecem de verdade. A descricao
da camara ja falava de algo que ninguem viu e voltou para contar; agora tem
gente de pedra no chao.

A sala VO15 saiu do banco: com a Medusa no objetivo, manter a mesma criatura
tambem no meio do caminho deixaria o grupo encontra-la duas vezes na run.

E, ja que agora da para prender o grupo inteiro de uma vez, a rodada que corre
sozinha (ninguem pode agir) passou de 3 para 10 voltas e avisa no canal se
ainda assim ninguem se soltar, em vez de parar calada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/planilhas/banco_vortice_oculto.xlsx
+++ b/data/planilhas/banco_vortice_oculto.xlsx
@@ -887,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1730,47 +1730,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>VO15</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Jardim de Estátuas</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Combate</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>As figuras de pedra no corredor estão em posições erradas: uma protege o rosto, outra corre. No fundo, algo se arrasta sobre a própria cauda e três vultos magros se levantam das sombras, farejando.</t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
-      <c r="M16" s="5" t="n"/>
-      <c r="N16" s="5" t="n"/>
-      <c r="O16" s="5" t="n"/>
-      <c r="P16" s="5" t="inlineStr">
-        <is>
-          <t>O que a última estátua ainda segurava na mão.</t>
-        </is>
-      </c>
-      <c r="Q16" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -1791,7 +1750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2159,114 +2118,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>VO15</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Nothic</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>1d10+3</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>VO15</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Medusa</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>3d8+3+2d6</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>172</v>
-      </c>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>Petrifying Gaze</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>O olhar endurece quem cruzar com ele.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>CON</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>